<commit_message>
Changes within nlp logic and repository structure
</commit_message>
<xml_diff>
--- a/data/url_data.xlsx
+++ b/data/url_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I185"/>
+  <dimension ref="A1:I205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7283,6 +7283,746 @@
         <v>5800000</v>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@productswithlanie/video/7476207587822685483</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> I spent $1500 at Sephora and I'm gonna show y'all what I got. So yes, your eyes are not deceiving you. These are, this is like, I don't even know how many bags this is, five? And then one big ass bag full of Sephora stuff. So, um, get comfortable because this is probably gonna have to be in two parts because we both know I talk a lot. So um, let's just get into it. $800. Oh my god. So starting off with this bag, we're gonna just pull out, I'm gonna need another 100% for her. Okay, so the first thing I got is this Benetint Cookie Highlighter. I've actually wanted this highlighter for a long time. I wanted it for Christmas but I ended up not getting it. But here it is, it's beautiful. The mirror's a little funny. But I love the Benetint Bronzer and one of their other highlighters that I have, but I've never got the cookie one so, finally got it. Next I got this YSL Love Shine Lip Oil Stick. This is the most beautiful color. I actually have it on right now. I put it on specifically for this video. This is the best lipstick, like lip oil stick that I've ever used in my life. Like the tart ones suck. The tart ones suck. So if y'all wanna get a lip oil, get this one. I know it's pricey but it's so worth it. Next is this Fenty Gloss Bomb. This is in the shade Fussy. I think this is like the basic shade, like it's the best selling but it's beautiful. It is beautiful. This shade is gorgeous and I don't like plumping glosses, like I hate them because they hurt like really bad. Like I don't know how y'all like those so much. So I just ended up getting the regular one. But I'm so happy I finally got one of the Fenty Gloss Bombs, like I've been wanting one for so long. Next is this brand new shade from Patrick Taw. This is She Goes to the Gym. This just came out recently and it's been out of stock in like every single store I went to. And then I finally found it. This is like the prettiest mauve color I've ever seen in my life. And these are like the most pigmented blushes I've ever used in my life. The most pigmented blushes. And the coloring is insanely gorgeous. Then we have this Dior, I think this is the foundation stick, yeah. This is the Dior foundation stick. I've heard so many things about this, about it being such a great base and everything like that. And I know a lot of like foundation sticks that just aren't good and then there's other obviously ones that are like amazing. So I'm really looking forward to trying this and seeing like how well it actually does work because when it comes to foundation sticks, it can go one of two ways, cakey or perfect. So I'm really hoping that this is not the cakey version, but we will find out. We had one more thing in this bag. This is the Dior Maximizer. I got this in the shade pearly. I tried on the pink one and it like evaporated. So I ended up getting the white. This is the pearl. This is basically like a liquid highlighter. I've seen people use this in their get ready with me's and it is beautiful. I tried this on the skin and this is the most beautiful liquid highlight that I've ever tried on my hand because I obviously haven't used it yet, but I cannot wait because it is so gorgeous and I love everything by Dior because they make some really, really, really good stuff. Like some really good stuff. Next is this bag. This was an online exclusive, so I did buy this online. This is the heavy cream from Fleur and when I tell you guys this literally smells like heavy vanilla whipping cream, I'm not lying. This smells so good. So good. I was like heavy cream. I really don't want it to smell like fresh cream from um philosophy, but no, this smells like literal vanilla cake batter cream. I love it so much. I should have gotten the big one because this is like the best gourmand spray that I've bought in a long time that just isn't spicy. Like this is truly gourmand. Next is this refi face sculpt lift and hydrate. This is the um the moisturizer and I've really wanted to like I've really been looking forward to seeing how this like works out because obviously right now I use the serif I moisturizer and this has like the balls on it to like, oh my gosh, like I. Refi has the best products ever. I use their um primer, best primer I've ever used in my life by the way. So I'm really really looking forward to seeing how this moisturizer. Yeah, I'm really looking forward to seeing how this moisturizer works out because I'm also a skincare girl. Next is this Natasha Denoa high glam concealer. This is in the shade RN1. I also have seen people say this is like the best concealer they've ever tried and my favorite concealer right now is the Huda Beauty matte one. So if this can top the Huda Beauty matte concealer then I will be I'll be sold because nothing right now is topping that concealer. So really hoping that this I have high hopes for this because obviously a lot of people say that this is the best concealer they've ever tried. So we will just have to find out. Next is this little like this is so cute. This is the cloud paint seamless cheek color from Glossier. This is in the shade puff. I don't remember the last time I used this type of blush. I think I was in like a junior in high school, but the color is so pretty. Well I would have shown you, but the color is so pretty. I used the tester in the store and it is the most like flawless pink finish. And plus this is just really cute. I think I'm gonna put this in my travel bag or something like that because it's really small, but I really do think that this would be like a really cute like summer blush color. And then lastly from that bag is the Glossier priming moisturizer. This is the most aesthetically pleasing looking package I think I've ever seen. See like that's the problem with me is like the packaging is like one of the main reasons why I buy so much stuff. Like if it has a pretty packaging I'm sold. So this and then plus it's a priming moisturizer so I feel like that'll kind of have a little bit of a similarity to the Bobbi Brown one, but I don't know. I love having a hydrated like base before I do my makeup so hoping that this does its job. Next bag. First what we have in here are these facial radiance pads. These are the glycolic and lactic acid face pads. Like they kind of exfoliate. I'm going to use them before I put any type of makeup on my face just to kind of get all that grossness off my face. I got the 28 pads just to test them out first because I'm not trying to get the $40 like 60 pads. That's ridiculous. So I ended up just getting the small 28 pads. This is from First Aid Beauty by the way. Next are these two products from Merit. This one is the priming or the. Oh I see the issue here. This one is the great skin priming moisturizer as well. I'm really starting to get into those though because I want to have a good base for my makeup and Merit has never seemed to disappoint me. So time to give this a try. And then we also got the the instant glow serum because obviously you put on a serum before makeup and then your moisturizer and then your primer. So I ended up just getting the matching serum to go with the moisturizer because I feel like you can never go wrong with having similar products because it reduces the chances of pilling. So next is this rare beauty melting blush in the shade Nearly Rose. I don't own that many cream blushes and when I saw this first of all hello when I saw this color I just immediately folded. This is the prettiest spring summer color I've ever seen in my life and rare beauty blushes are already on top. So I figured let's just try a cream blush by them. See how it goes. Next we have this Rify gloss highlighter. I've also heard many good things about this. This is like the this is in the shade I think it's only one shade but Topaz it's like a kind of the same thing as the blush from Glossier. I actually don't use that much liquid highlighter so I feel like if I put this on before the powder highlighter it will turn out really really really pretty. Plus you can never go wrong with Rify. Like hello their products are absolutely beautiful to die for. Come back for part two because I'm running out of time.</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>productswithlanie</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>126200</v>
+      </c>
+      <c r="E186" t="n">
+        <v>141600</v>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">biggest haul i’ve ever done. part 2 coming soon 😋 #fypage #fypシ゚viral #fypシ #foryoupage #foryou #viral #foryoupage❤️❤️ #fyppppppppppppppppppppppp #f #fyp #hygiene #hygieneproducts #hygieneroutine #hygienetok #bodycare #bodycareroutine #bodycareproducts #beauty #beautyproducts #beautytok #makeup #makeuphaul #makeupmusthaves #makeuptok #sephora #sephoramakeup #sephorahaul #hugehaul #haul #haultok </t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr"/>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>2025-02-27</t>
+        </is>
+      </c>
+      <c r="I186" t="n">
+        <v>881100</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@danielaavillam/video/7451358007214001441</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Haldesefra Express porque me viene a recoger en 10 minutos. Me he dejado un poquito de dinerit y les voy a enseñar la que me he gastado, ¿vale? Porque me hace mucha ilusión. Hace unas semanas me cogí la crema de Inkey List de que lleva... no me acuerdo que lleva, la noboretín o algo así, para los granitos y me ha funcionado súper bien porque me ha comprado los brotes de granitos por la regla y me ha quitado mucho. O sea, estoy muchísimo mejor y estoy súper contenta. Y ahora me he cogido este serum de Neacellamida de De Ordinari para controlar las manchitas, para intentar reducirlas un poco. El Brow... Olé. El Fluff Unfixed Brow Watch Serious Urges... El gel de cejas de sefora nuevo que lo he visto por TikTok y va súper bien. Vamos a verlo. Yo creo que está bien. Estas gotas broncedoras de Islet of Paradise que he visto que están muy bien y hacen la competencia de las de Drunk Elephant. Vamos a ver, vamos a elevar un poco este color de palita que tengo que parece el de la camiseta. A ver, a ver qué tal va. Una de las cosas que más ilusión me hacen, la Magic Cream de Charlotte Tilbury. Yo la he probado, pero la he probado en mano. Espero que las sensaciones sean la misma en la cara. O sea, es que me encanta. Me encanta y me hace mucha ilusión, pero a la vez me da un poco de miedo porque como me encante y me quiera coger el grande... Bueno, bueno. Piano, piano, piano. De esta siguiente cosa tiene la culpa la María. Sí, María, tienes tú la culpa. Y me la he cogido en mini porque sé que me encanta y me la he probado ya y yo quería la grande, pero es la última cosa que cogí y dije, amore, era ya mucho cheles. Así que me cogí en la pequeña primero. Sé que la voy a gastar en nada porque la voy a usar para cada día porque el efecto que deja es el que quiero diario y las deja preciosas. No es que de volumen te las curva y te las deja como súper estiradas y como definidas. ¿Sabéis lo que quiero decir? Ya me entendéis. Sé que me entendéis. Una cosa que me hace mucha ilusión es el gloss de Jisoo, el Strawberry, pero sin glitter porque han sacado uno nuevo, creo que es por Navidad, que lo he visto en tienda que es con glitter y este es el normal. No es mate porque es un gloss, pero no tiene glitter. Sé que me entendéis. Yo sé que con mis explicaciones, aunque sean pésimas, sé que me entendéis. Se lo vi a Rocio, ¿lo ves qué se llama? Bueno, una chica de Instagram que me encanta y es como así, muy blanquita como yo y con ojos claros y le quedaba monísimo. Me probé en tienda el de mango, que es como más naranja y no me gustó nada. O sea, no me quedaba nada bien. Así que creo que este me quedará súper bien y es monísimo para día a día. Otra cosa de skincare es la Drain Solution, que me quería bajar la de Mario Badescu, pero me han dicho que estaba súper bien también y más barata. Así que vamos a ver si funciona. Eso es para los spots. Por ejemplo, ahora estoy granito, pues me lo pongo y se seca. ¿Sabéis? Y eso en vez de los gummets. Ya sé que hay gente que es muy fan de los gummets, pero a mí no me gustan nada. O sea, se ven. La gente dice que no se notan, pero se ven. Y a mí no me gustan, sinceramente. Bueno, para gustos colores, ¿no? Primero, me voy a enseñar una cosa que no me hace tanta ilusión. O sea, que sí que me hace ilusión porque me encanta que lo me cogíes y no me lo hubiera cogido. Pero eso lo voy a dejar al último. Me he cogido otra vez porque me regalaron por mi cumple mis amigas el set este. Y bueno, lo tengo. El armario está súper desordenado. Bueno, no lo voy a enseñar, que lo tengo por ahí. Me lo pongo cada día todo. Bueno, el gel no. O sea, qué ha parecido que no me ducho cada día. Me ducho cada día, pero no me lo uso cada día porque como es muy pequeño no quiero gastar tanto. Pero bueno, eso me está acabando todo. Bueno, esto se me ha acabado. Eso me está acabando y esto también. Que lo he repuesto, vamos. Ahora sí que sé. Me he cogido los polvos sueltos de Huda. Obviamente me he cogido el tono Cherry Blossom porque es la mejor calidad que la camiseta. Ya lo he dicho. Y yo creo que he estado dando entre estos los pound cake, que creo que son como los dos los más neutros antes del blanco. Pero no, el Cherry Blossom porque son los que los únicos que he probado, los del Arnau y los de la Miriam, que los amo y me encantan y los quería. Así que además ellos los tienen porque los hemos cogido por cumpleaños. Así que yo los necesitaba. Y ya está. Lo que yo he tenido que hacer un cambio, porque ayer dije sí, es esa cesta que lo dejé en caja. Y no sé por qué puse sin querer el aceite de Shisou también de pelo, pero el grande. Amor, 40 pavos creo que valía. Y dije, luego llegar a casa. Esto no es mío, cabrín. O sea que supongo que lo habré puesto pero sin darme cuenta. Y pues he vuelto porque yo quería este. Y pues lo he cambiado. Pero claro, luego, o sea ahora llegar a casa, después de haberlo cambiado, he dicho, será una señal del universo en plan el universo quería que me lo cogiera. A lo mejor lo necesito. Lo veremos en los siguientes capítulos a ver si lo compro.</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>danielaavillam</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>415</v>
+      </c>
+      <c r="E187" t="n">
+        <v>3797</v>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">que es lo que mas os gustaaa?? q hago cojo el aceite de gisou tambien???!!! ayuda chicas funciona?? #sephora #sephorahaul #theordinaryskincare #theinkeylist #hudabeautyeasybake #parati </t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr"/>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>2024-12-22</t>
+        </is>
+      </c>
+      <c r="I187" t="n">
+        <v>41600</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@andreagarte/video/7351146220024319265</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Lo de gastar todo tu dinero en Sephora es una obsesión y es la mía. Pues voy a enseñar todo lo que hay aquí dentro. El Milk Monsterizer Cleanser de Bayomo. No sé nada de él, lo tendremos que probar. Gel de Cera D anti-intersecciones, este de aquí. Unos parchecitos para los ojos. El de Befoon, de Valentino. Este Chameleon, este que es. Cleanser de Bayomo para viajar. Un poquito de Olaplex número 7. Las drops de Nia Jaramina de Sandia, estos de acá. Qué ganas de probar esto. El de The Professional, este de aquí, es un limpiador que amo. De Valentino también, pero para hombre, para Víctor. Vamos a ir igual a este parche. No tenía yo un blast de Red Beauty. Ahora ya sé. De mis parches fabs para los ojos, estos de acá. Una cremita en tamaño mini también de viaje. La máscara de pestañas de Tarte. Se nota muy pesado el packaging, creo que esto me va a encantar. La Bora Butter Repair Cream de Drunk Hallow Hand. Amo estas cremitas de Pulsar. Bronzer en talla mini de Milk. Para mi neceser de viaje, mira esto. Más mini tallas para mis viajes con este mini neceser de Yves Saint Laurent. Miren este labial. Mira esto. La máscara de pestañas L'Asclas, también en formato mini talla. Súper chiquitita, me encanta. Y un perfume de viaje de Yves Saint Laurent, libre. Huele increíble. Lo tiro todo. De reposición, el Benetim de Benefit. Amo esto para dar color a mis mejillas y labios. Es lo mejor. Mulsterizer Hair Cream de By Oma. Chiquitita. Labial de Sephora de estos que me gustan a mí, que son muy nude. Esta pedazo de caja de los barritos de Sephora. La cual estoy deseando abrir. ¡Clara! Hay muchas cosas aquí dentro. Este labial de Make Up by Mario, que son de los que se giran y son como un blush. Esta máscara de pestañas que me encanta. Un lápizito en este tono rosita. De Rare Beauty, este lápiz de labios en este tono que, sin duda, son mis tonos. De Illya, por aquí tenemos este blush en gremita. Y de Milk, también en formato un poquito más grande. El contorno. Para terminar, iluminador de Rare Beauty. Bueno, pues no me queda nada más que añadir, la verdad. Nos vemos en el próximo vídeo.</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>andreagarte</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="E188" t="n">
+        <v>6303</v>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>MEGA HAUL de @sephora ❤️‍🔥</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr"/>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>2024-03-27</t>
+        </is>
+      </c>
+      <c r="I188" t="n">
+        <v>94800</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@katiefanggg/video/7470675926695578935</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> It's time for a Sephora haul. I feel like I haven't done one of these in forever, so I'm excited. Okay, first, I actually got these in PR, but I wanted to show I got the little, like, blush things from Gloresky, and they're so freaking cute, and I'm so excited to try these. And then Summer Fridays sent their new, like, birthday bomb, and the packaging is so cute. Okay, let's get into the actual stuff that I bought. Okay, first thing I got is the Color Wow Extra Large Volumous Spray, because when I do my blowouts, I like my hair to be, like, really big. And I love my, um, living proof one, but I wanted to try this because this is, like, a mousse, so. Okay, then I got the new Gisu Hair Mask. I've been really into, like, hair masks recently, and I always give mine away, so I was like, I might as well try this. Look at how cute the packaging is. It's, like, honey, and it smells so freaking good. But yeah, I'm really excited to try this because my hair needs help after Fashion Week. Okay, next I got two of these Rare Beauty eye patches. These are so good. I love the Peter Thomas Ruffles one, but these are my second favorite. They, I don't know, something about them is just so good. And they come in little, like, packs like this, and they're great for, like, traveling, too. I don't know, it just feels, like, really nice and refreshing under the eyes, so restocked on these. But yeah, this is, like, my fourth or fifth bottle, which is kind of crazy, but that's how you know what's good. Okay, again, didn't purchase these, but I wanted to mention Rode saw my video and saw that I was running low on my cleanser. They sent me a restock of the pineapple one and then a little mini version, too. So sweet of them. And then I got a restock of my lip liner from Makeup Forever. This is in the shade Wear a Real Walnut. SUNY inspired me, but yeah. And then more stuff for my hair because it'd be getting crusty. This is the Moroccan Oil Treatment, and I've heard, again, a lot of good things about this. I'm pretty sure my mom uses this, too. Oh, this is the bottle, and it comes with a little pump. So yeah, I'm excited to use this. And then I got... I keep losing this. This is my favorite eyelash curler, and it's just, like, I bring it everywhere with me, and that's probably why I keep losing it. But this is the best eyelash curler in the world. Oh, and I just wanted to show this, but Laneige sent me their new, like, lip thing, and it's so good. Like, the cushion thing on your lips, it feels so good, and I love it. And that was my Sephora haul. Anyways, yeah, bye.</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>katiefanggg</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>6200000</v>
+      </c>
+      <c r="E189" t="n">
+        <v>256400</v>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Love me a haul</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr"/>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>2025-02-13</t>
+        </is>
+      </c>
+      <c r="I189" t="n">
+        <v>1800000</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@julia.reverte/video/7460976620933860640</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Ayer fui a los cojos, solo me tenía que comprar una base, pero fui con una amiga que le ganaba maquillaje y me empezó a recomendar cosas, entonces pues bueno, me las compré. Y os voy a enseñar. Vale, la base, la Estee Lauder, el tono 2D1, que es la que yo utilizo. Para mí es la que mejor me va. No he probado muchas de bases, pero antes me salió como un brote de acné hace unos años y la probé y es la que más me tapaba. Entonces ya me quedé con esta, pero a mí sí que me da mejor. Luego me compré el bronceador de Charlotte Tilbury, que he visto que lo tienen todas, me ha ganado súper bien. Y yo tengo este, que vale 3 euros, es lo primero que cogí un día que dije necesito bronceador, no tenía, fui y cogí esto y me saca granos. Entonces, ¿qué pasa? Pues me lo cogí. Después, no podía faltar los polvos de cuda, hacía tiempo ya que los quería. Me cogí los Cherry Blossom K, para mí son los que mejor me van, porque mis amigas tienen diferentes tonos, entonces me los he probado. Y los roses son los que mejor me quedan, me ilumina un montón. Luego, esto ya creo que me lo compré en Drunie. El Rimmel este, porque yo tengo este, pero si me disparce todo por aquí, no sé por qué. Entonces pues cogí este que es waterproof y si salgo de fiesta, pues este y de normal, este. Cogí esto para el pelo, que es un protector térmico, es mejor que he probado, la verdad. Vale, por último, esto que es un fijador, porque me iba a comprar el de Charlotte, pero mi amiga me dijo, tengo este y el de Charlotte, iban igual, deberían los dos. Entonces pues dije, como es más barato, pues cojo este. Y ya está, y suerte que sólo iba por la base.</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>julia.reverte</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>558800</v>
+      </c>
+      <c r="E190" t="n">
+        <v>13700</v>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>són 4 cosas pero me he dejado medio riñón 😂</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>2025-01-17</t>
+        </is>
+      </c>
+      <c r="I190" t="n">
+        <v>177400</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@albadlcruz/video/7473066872410230038</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Yo me acabo de ahorrar 62 euros de mi wishlist. Esto es muy heavy. Te voy a enseñar el pedido que yo he hecho. Es que sabéis que normalmente no suele entrar tart, así que he aprovechado y me he cogido el corrector de tart en formato mini para utilizarlo como base de sombras. Voy a ir de viaje en unas semanitas y lo voy a necesitar, así que así lo pruebo. También he pedido el mini del Hollywood Flows Filter de Charlotte, pero en un tono más oscuro para poder mezclarlo con la base, para utilizarlo como bronceador. No sé, a ver qué tal. También he pedido el mini de los polvos compactos de Charlotte, que sabéis que son mi vida entera. Los utilizo muchísimo para la zona de la ojera. Como me voy de viaje, de nuevo me lo he pedido para poder llevármelo. Yo iba haciendo alojitos al bronceador de aorulas muchísimo tiempo. Sabéis que tengo la paleta que viene en seis, pero quería tenerlo aparte para poder llevarmelo sin tener que llevarme la paleta muchas veces. He cogido el tono nude bronze light a ver si no me queda naranja. He cogido también el mini gloss de Fenty en el tono Fuzzy, porque muchísima gente ama el tono Fuzzy y yo no lo he probado, así que pues era mi oportunidad perfecta. Y por supuesto, uno de los nuevos colores de Deep San Logan, o sea, el tono Berry Bang. De ser más bonito el tono Berry Bang. Estoy obsesionada con los colores Berry últimamente. Skin tint de Hourglass porque necesito probar esa maravilla. O sea, yo cuando se lo veo a las chicas les veo ese look tan bonito que ese maquillaje estaba en mi wishlist hace muchísimo tiempo y como que no me animaba a cogérmelo. Espero haber acertado con el tono porque últimamente no estoy muy fina yo con estas cosas.</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>albadlcruz</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>105200</v>
+      </c>
+      <c r="E191" t="n">
+        <v>724</v>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Respuesta a @Noelia esta es mi compra en Sephora para aprovechar el 25% de descuento 🫣❤️‍🩹  CÓDIGO: ALBA (afiliado) - es el mismo que el que ofrece Sephora en su app.  #makeup #maquillaje #sephora #sephorahaul #wishlist #makeupwishlist #rebajassephora </t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>2025-02-19</t>
+        </is>
+      </c>
+      <c r="I191" t="n">
+        <v>17100</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@ainhoahumet/video/7473235984403139862?_r=1&amp;_t=ZG-8uFLVIuwuMy</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr"/>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>ainhoahumet</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>6524</v>
+      </c>
+      <c r="E192" t="n">
+        <v>18900</v>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Respuesta a @charli 💘 haul de sephora nueva york💓🇺🇸 seguramente el más grande de mi vida, que ilusión!! 🥹 #haul #sephora #haulsephora #maquillaje #parati </t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>[WinError 123] El nombre de archivo, el nombre de directorio o la sintaxis de la etiqueta del volumen no son correctos: 'C:\\Users\\sandr\\Documents\\scrp_tiktok_tfg\\videos\\7473235984403139862?_r=1&amp;_t=ZG-8uFLVIuwuMy.mp4'</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>2025-02-19</t>
+        </is>
+      </c>
+      <c r="I192" t="n">
+        <v>165400</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@andreacarpn/video/7474975205035740438</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Si pudiera volver atrás, ¿cuál sería mi primera compra en Sephora? Los productos que considero que son más clave y esenciales y sobre todo super fáciles de utilizar Sabía yo que esto no iba a salir bien En primer lugar tenemos el contorno hidratante de Milk y es que este producto para mí, aunque parezca un poquito caro, viene muchísima cantidad Yo lo tengo desde abril del año pasado, lo utilizo todos los días y mirad por dónde va el producto y es verdad que probo alternativas locos y no me han acabado de encantar Seguimos con un buen corrector Tengo este que es el Radiant Creamy Concealer de NARS Tiene cobertura media, super ligerito para la zona de la ojera Pero de eso tenéis varios correctores en función de lo que busquéis Por ejemplo el de Too Faced está super bien si buscáis una alta cobertura pero sobre todo que os hagáis con un buen corrector Y siguiendo por esa línea Estos polvitos de huda Es un producto que cunde un montón A mí los tengo desde abril del año pasado y los utilizo todos los días Y es que para mí no hay polvitos de sellar como estos Seguimos por este combo de mejillas Es el nuevo contorno barra bronceador en líquido de Rare Beauty y uno de sus colores Son super cremosos, super fáciles de trabajar y super modulables Y por último este bronceador de por aquí que es el de Too Faced Es que mirad que tono tan bonito Y sí que es verdad que cuando yo utilizaba otros más low cost costaba mucho más trabajarlos, eran más sequitos La duración también se nota Y nada, esta sería mi selección Y lo que os aconsejo 100% es que si queréis coger alguna cosita en séfora esperéis a que haya algún descuento Rare Beauty no suele entrar en este tipo de ofertas Pero bueno, el resto sí, así puedes conseguir los productos un poquito más baratos</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>andreacarpn</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E193" t="n">
+        <v>778</v>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mis imprescindibles de Sephora, tenéis hoy un 25% de descuento en la app!!! #sephora #sephorahaul #sephoraspain #makeup #maquillajedealtagama #fyp </t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr"/>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>2025-02-24</t>
+        </is>
+      </c>
+      <c r="I193" t="n">
+        <v>11000</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@nats_not_okay/video/7400145747280448814</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Hey guys, okay, so I just got done Shopping at Sephora and I did some major damage and I wanted to show you guys like what I got These are a few things that like maybe I had heard about from somewhere or like maybe seen a video on once and I was Just like yeah, give it to me. Let's try it starting off insanely strong. I have the wow dream coat I believe this is that yeah, this is the extra strength one. I've been wanting to try this so bad I use the dream coat back in the day and I liked it I've been wanting to try this for a while now and I've been wanting to try it for a while now and I've been wanting to try it But I heard the extra strength is really good for girls with like a little bit of curl or like wave to their hair and My natural hair has like a little bit of a wave to it. Also like all for trying new foundations This is the makeup forever HD skin Hydra glow foundation and I got it in the shade 3n40 I've just heard it's supposed to be like really lightweight and I'm gonna see if a product can do both of those things at the same time next, you know her you love her This is the Fenty Beauty Kilowatt freestyle highlighter duo. This is the shades ginger binge and Moscow mule This is the one that notoriously Madison beer uses and has like sworn by forever Anything Madison beer does like I'm sad. I can't wait to try this on my actual cheeks But when I swatched it I was like X y'all know how I love say and like literally all of their products They're all so dewy but this is the say do bronze soft focus liquid bronzer and I got it in the shade swim I kind of just like eyeballed my shade. I didn't even really like swatch these It's just supposed to be like really lightweight like really hydrating and just a good little like dewy bronze on the skin I also got a mascara which if y'all know y'all know, I love my lashes, but I'm trying to become a mascara girly I feel like I'll be more compelled to just wear a mascara if I get a mascara that I really love Y'all also have any other mascara recommendations? Let me know cuz your girl is in the market and I'll let you guys know how I like this one, too This product I'm really excited to try because when I put it on my skin in the store It was like so tacky and I love that This is the Anastasia Beverly Hills brow freeze gel now We all know the brow freeze in the little pot and I like it But it really didn't hold my brows that well now to be fair Like I haven't gotten my brows done in literally like four years, which sounds insane. I just like upkeep them myself I really want to get a product that's going to hold down my brows and this just kind of caught my eye I hadn't really heard anybody talk about it. This was marketed as like extra hold So when I hear extra hold I'm thinking like hairspray for my eyebrows, okay This is the NARS creamy radiant concealer. We all have so much respect for her. This one's not like a product I haven't tried before I literally have this already in three different shades, but I wanted to get another shade But we'll see how it incorporates and like mixes with my current products that I've been using So you never know this is the freck XL pin A lot of you guys always ask me about my fake freckles and like what product I'm using and it's always the freck XL pin I swear by it. I think this last one that I just ran out of I got like Three almost four months ago like the beginning of summer and lastly but certainly not least I finally broke y'all. This is the Patrick tall all over face and body glow bomb in the shade She's on vacation. I'm always tempted to buy it and then I feel like every time I actually want to buy it It's never in stock. So I finally got it. I love my soul de género So I'll be interested to see if this will pull me away from her But I have heard people literally rave about this forever Really did my big one on this one literally did her big one me with the leah vocal stems recently hot girls Love leah hot girls of PPG hot girls love leah serena and janay period. But yeah, that's everything Love you guys</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>nats_not_okay</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>372900</v>
+      </c>
+      <c r="E194" t="n">
+        <v>57900</v>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEPHORA SUMMER PRODUCTS HAULLLL 🌊🐚✨ hope yall enjoy bc my pockets hurt HAHH #fyp #haul #sephorahaul #makeupinspo #beautytok #summermakeup  @Color Wow Hair @makeupforever @Fenty Beauty @Saie @meritbeauty @Anastasia Beverly Hills @NARS Cosmetics @Freck Beauty @Patrick Ta Beauty </t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr"/>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>2024-08-06</t>
+        </is>
+      </c>
+      <c r="I194" t="n">
+        <v>535000</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@beautygossipp/video/7471184669321481494</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Economizando Séfora para tener más productos por menos dinero. Para ello te tienes que ir directa al stand de los productos mini talla, porque estos que te voy a enseñar sí que merece la pena comprarlos en versión mini. Primera parada a los polvos de Huda Beauty porque son buenísimos, además de pequeños porque te los puedes llevar a cualquier lado y duran mucho. Luego un clásico que son los coloretes de Rare Beauty que aunque sean minis nunca se acaban. Otro productazo que es el corrector de Nars que de normal cuesta 30€ pero en esta ocasión 18€. Y de la misma marca tenéis tanto el colorete como el bronzador que estoy enamorada de ellos porque son super minis y caben en cualquier lado. También está el famosísimo gloss de Jisoo por 26€. Y para terminar aunque hay muchos más productazos, este contorno de Tarte es muy mini pero cumple su función y además se difumina que da gusto. Tenéis más opciones en versión mini para elegir. ¿Queréis parte 2?</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>beautygossipp</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>1207</v>
+      </c>
+      <c r="E195" t="n">
+        <v>10900</v>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Economizando Sephora: + productos - dinero 😊🙃 Los que te enseño son mis favs🥴 ¿Team mini tallas o prefieres el full size? 👀👇 #sephora #sephoraminis #sephorahaul #mini #makeup #maquillaje #beauty #rarebeauty #contentcreator #makeupaddict #parati </t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr"/>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>2025-02-14</t>
+        </is>
+      </c>
+      <c r="I195" t="n">
+        <v>130800</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@oliviamassucci/video/7475050420935642411</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Sephora haul featuring some of the things you guys influenced me to get which thankfully de-influenced a lot because somehow all of this was still almost $300. I don't know either. Let's get into it. Starting off with the new items, the Charlotte Tilbury glow foundation stick. This is all over my for you page so it's about time I try it. I really hope I got the right shade. I also want to do a video of my first impression on this. I feel like it's gonna be really pretty. I literally cannot wait to use it. Next we have the Kerastase premier oil which I did actually already use. I use it today and my hair feels really good. I usually use Kerastase gold elixir one. This one's really good for split ends specifically and I've been dealing with that a lot so trying this can fix me. I'm so excited for this. This is the Dior backstage glow palette. One of my most influenced that you guys said. I really don't think you're gonna let me down because it looks stunning. It's actually breathtaking. I don't even want to mess it up. I think I'm most excited for the bronzer part. Let me know in the comments which one your favorite is. Now for some things I just wanted to restock. Love the Glossier skin tint. It's just so light and so natural so moving into spring and summer. This is an essential. You guys know I cannot live without my Cosas brow duo. This is their brow pencil and then their brow gel. It's literally the best brow gel I've ever used. The color on it is amazing and I swear it stays all day long. I cannot wait to use everything.</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>oliviamassucci</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>990500</v>
+      </c>
+      <c r="E196" t="n">
+        <v>2195</v>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loves a good Sephora run 😙😙 #makeup #beauty #sephorahaul </t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr"/>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>2025-02-24</t>
+        </is>
+      </c>
+      <c r="I196" t="n">
+        <v>28600</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@krissyg_95/video/7476338584635657494</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Guys I went to Sephora and I'm hoping I found my new favorite lip combo. I don't actually have one that I really stick with so let's see maybe this is what it is. I've just got a lip liner on and I bought this lip balm in birthday cake. It's actually really nice and it lasted really well. I had it on for like a few hours. I'm gonna take this off and let's see. I've got a new foundation. This is the foundation that I wear in shade Barcelona when I'm tanned and I mix it with the Estee Lauder lipstick. Finally I got hold of this gloss. I think I've been to Norway, Venice, Sephora and everywhere sold out. I got this lip liner because I swatched it and I swatched like loads of lip liners and then when I went to wipe it off there was one that didn't come off like literally didn't come off and I was like which one was that so I spent like half an hour on the store looking for this because I forgot what I swatched. I do it all the time like I swatch stuff, walk away and then if you go to remove it or like you look at it again maybe like a gloss and it looks actually decent and then I also got just the Sephora gloss. This looked really nice on my hand. So the lip liner is Make Up For Ever in this shade. It's this Artist Colour Pencil Extreme and this is in the shade Endless Cacao. I do like a really dark liner. That's like usually my go-to. So creamy like then for lipstick I swatched this I wasn't gonna get it then I walked away and like I said I was like oh this is actually really nice I forgot which one that was so this is Fenty Gloss Bomb Sticks and this one's in the shade Blaze Donut. Let's try hmm I don't know if I've gone too cold tone with my I'm gonna add a little bit of the Golden Girl by Dole Beauty just because it is really really nice. I'm gonna add a little bit of the I'm gonna add a little bit of the Golden Girl by Dole Beauty just because it is really light and I feel like because the liner is so dark this is what it's looking like I do like it then to finish off which is obviously the best bit is gloss and I've been dying to get hold of this this is the Huda Beauty in Sugar Baby. This shade is never in stock and my go-to is like I said is dark lip liner really light lipstick and then a pink gloss and this is the perfect definition of pink pink that is that is perfection I do like it this is my definitely maybe I'm not in love with the lip line I'm not gonna lie I probably will maybe try this again and see how it wears or maybe I just need to get a different because I did get a really cool tone and it's just looking a little bit grayish when I put it on so I might either try a different one but I do really like the lip combo the gloss it's staying it's probably going to be my new favorite the it's this one's also very similar to the Huda Beauty and it has like a really nice shimmer on it as well so yeah if you ask this is the lip combo that you guys always ask this is probably gonna stay for a long time but I do switch it up all the time so honestly I never know which one I'm wearing</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>krissyg_95</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>895400</v>
+      </c>
+      <c r="E197" t="n">
+        <v>30100</v>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mini Sephora haul #sephora #lipcombo </t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr"/>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>2025-02-28</t>
+        </is>
+      </c>
+      <c r="I197" t="n">
+        <v>1400000</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@ssofimakeupp/video/7222411930152062214</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Mirad lo que tengo. Yo no me pude resistir y he comprado todas las cosas más virales de TikTok. Vamos a verlo. Yo no sé cuánto tiempo llevaba queriendo este producto y evidentemente es el Hollywood Flawless Filter de Charlotte Tilbury. No os imagináis las ganas que tengo de probar esto, o sea, me muero de la ilusión. Me lo cogí en el tono 3 porque, bueno, yo soy bastante blanquita, así que... Lo siguiente también se hizo super viral y son los nuevos coloretes de Too Faced. Yo fui a la tienda a mirar un poquito y mi tono favorito fue este de aquí, que es el Velvet Crush. Voy a meterle el dedo en directo. A mí me encanta este tipo de tonos. Yo me lo probé en la tienda y dije, este tiene que ser para mí. Además, es que mirad, qué mono. Me explicáis las ganas que tenía yo de probar la marca Ren Beauty, que para quien no lo sepa es la marca de Ariana Grande. Y obviamente tenía que pedirme una de sus sombras líquidas. Estáis viendo este color. Y mirad qué preciosidad. Yo no puedo. Más productos de mi queridísima Rihanna. Por si no lo sabíais ya, es mi marca favorita. Y yo no sé por qué todavía no tenía esta base de maquillaje, la Ice Drops. Es super viral en TikTok y yo ya la he probado, me encantó. Y dije, la compro ahora. Es en el tono 3 y ya os digo, ya la he probado. Me ha encantado esta base de maquillaje y la necesitaba comprar para mí. Y lo siguiente son los nuevos polvos compactos. Que por cierto, mirad el packaging, qué chulo es, porque no sé. Viene con esta esponjita de aquí. Y yo no sé si soy la única que lo piensa, pero tiene un ligero tono rosita. Así que ya veremos qué tal, pero vamos, que seguro que viene. Me mandaron de regalito esta muestra de aquí del Fenty Glow, que es uno de sus glosses más virales. Estoy deseando probarlo. Y ya de muestritas me han mandado la Skin Hero Peeling de Herborian. Y obviamente una muestrita de perfume de Dior. Así que estar muy atentas porque obviamente esto lo tenemos que probar juntas.</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>ssofimakeupp</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>119000</v>
+      </c>
+      <c r="E198" t="n">
+        <v>19500</v>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adoroooo todas mis cositas nuevas de @SEPHORA España ❤️‍🔥✨ #sephora #sephorahaul #comprasmaquillaje #makeup #makeuptutorial #makeuphaul #sephoragiftlist #altagama </t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr"/>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>2023-04-16</t>
+        </is>
+      </c>
+      <c r="I198" t="n">
+        <v>302200</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@eugeniardzc/video/7304008564253674757</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Hoy les tengo un haul de Sephora. Me estoy llegando de San Antonio y compré un chorro de maquillaje. Y compré mucho del maquillaje que ya tenía. Porque como me ha tocado viajar mucho por trabajo, cada semana me tardo como una hora en empacar mis cosméticos. De verdad, siempre pienso todo. Así que dije, ¿sabes qué? Voy a hacer una cosmetiquera de viaje. Me compré la famosísima Matt's Palette. Y me compré dos delineadores. Uno es el Daniel, que es mi color favorito, y el Angela, nunca lo he usado. Me compré el Blush Stick de Makeup by Mario en el color Earthy Pink. Es este color que me encantó, no lo había visto. Y atrás, tiene una brochita. De Hourglass compré un chorro de cosas. Y les voy a hacer un review usando todo porque nunca he probado nada. Me compré este Voolumizing Glossy Balm. Me los compré en diferentes colores. En Scents, en Sleep y en Mist. Estos son los colores que he visto virales por todo TikTok. Me compré esta Foundation Brush, que dicen que está buenísima. El Airbrush Concealer, también vi que está wow. El Finish Concealer Brush, para el concealer. No me lo compré, no me acuerdo. El Foundation Stick de Contour. Y por último, el Ultra Sleep High Intensity Lipstick. Uno que es lo que me ama. De Charlotte Silbury me compré el Sitting Spray. Para mí, cosmetica era doble. Y este también, que es el Matte Bronzing Filter. Que me encanta, que también es doble para mi cosmetica. De Rare Beauty volví a comprar mi base para mi cosmetica. Era doble. Y es el color 210N. Me encanta esta base, es la que tengo puesta ahorita. Y me compré el Hope y el Virtue. El Hope no lo he probado, el Virtue ya lo tengo. Y también este que me encanta. Que es el Base Luminating Primer. Estos de verdad tengo miles en mi casa. Pero siempre compro porque los amo. Y es la primera vez que encuentro el Menta. Así que lo pondré a prueba. Amo los de Summer Fridays. Me compré el Setting Powder de Laura Mercier. El nuevo que es el Ultra Blur. Para probarlo en grande y en chiquito. Amo este powder así que no creo fallarle. Encontré la marca Refi. Y me compré el Cream Bronzer para probarlo. El de las Brow Sculpt. Que es el mejor para la ceja. Y este cual es? Ah, el Lip Sculpt en Rosewood. Que me encanta. Compré el otro blush que me encanta. Es el 001 Pink. Es mi favorito. Y volví a comprar un Gloss. Que este es el Rosewood. Me encanta. Y compré estos highlighters. Que moría por probar. Os voy a enseñar. Vean la belleza de este highlighter. De Patrick Tau. Me compré la palette que se llama Major Eyeshadow Palette. De verdad los empaques de Patrick Tau. Son otro nivel. Se me hicieron increíbles los colores. Y me compré el She's That Girl. Ya tengo varios para probarlos con ustedes. Y decirles cual es el blush que más me gusta. Me compré una blotchita. Y el Fancy Gloss Heat Bum. Era un Chocolate Lipstick. A ver como me queda. No es mi color favorito. Pero lo vi y me gusto. Eso es todo.</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>eugeniardzc</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>436000</v>
+      </c>
+      <c r="E199" t="n">
+        <v>58400</v>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mega sephora haul! De verdad alguien me tiene que poner un alto que amo el maquillaje jajajaja😮‍💨🫢 díganme que otros productos me recomiendan y si hice buenas compras #makeup #sephorahaul #makeuphaul #sephora #shopping #foryoupage </t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr"/>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>2023-11-21</t>
+        </is>
+      </c>
+      <c r="I199" t="n">
+        <v>563300</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@jirethmerchan/video/7376031594684927264</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Si vas por primera vez a Sephora a comprarte maquillaje de alta gama, mira este vídeo porque te voy a dar mis recomendaciones que me gustaría que me hubieran dado para comprármelas el primer día que fui a comprar en Sephora. Sin duda, como basta mi maquillaje favoritísima de este año y mi gran descubrimiento, la All Hours de Issa Laurent, es como que te deja un acabado mate, pero es que es muy hidratante. Si tienes la piel un poquito más seca, la de Luminous Silk es una pasada, o sea, súper hidratante, te deja la piel un poco blue, o sea, es una maravilla. De correctores, el más hidratante para mi parecer, el Dior Forever, es una maravilla, cubre muy bien, pero es que a la vez es como muy hidratante, no sé que te cuartea la ojera, te dura todo el día y si quieres algo que más te cubra, o justamente para el párpado o para las sombras porque pigmentan un montón, el de Huda Beauty, es que esto te cubre tu pasado más oscuro. Os lo juro, es un corrector que lo utilizo todos los días. Hoy sí que es verdad que llevo esta porque quería algo más ligerito. Como bronceador en barra, te recomiendo muchísimo el de Sephora Collection si tampoco te quieres gastar mucho porque el de Make Up by Mario está muy bien y el de Rape Beauty también, pero sí que es verdad que este, me parece muy buena comparación al lado de los otros, es una maravilla. De polvos sueltos, obviamente estos de Huda Beauty no te van a decepcionar, son una maravilla, vienen en 8000 tonos, son súper ligeritos, te dura 4 vidas, o sea, no ha pasado. De bronceador en crema, sin duda, Charlotte Tilbury, o sea, es que este se lleva el premio al mejor bronceador en este formato, es una maravilla. Este es el tono 1, lo noto como más frío, está entre frío y cálido, o sea, no es ninguno de los dos, pero bueno, si queréis ese efecto de bronceado pero contorno a la vez, este está muy bien y si queréis algo más bronceado, el tono 2 está genial. Iluminador, sinceramente, obviamente, la paleta de Dior, este el tono más clarito, da igual, es que esto es una maravilla, es que no lo dejo de utilizar todos los días, es una pasada. De colores en polvo, te recomiendo muchísimo los de Too Faced porque viene bastante cantidad y es que esto no se me acaba nunca, aparte pigmenta una brutalidad. Es verdad que a mí el olor personalmente no me gusta mucho y esto os lo digo para que lo tenéis en cuenta, no me gusta mucho, pero es que el productazo es una maravilla y me compraría de todos los tonos. También como otra alternativa tienes el de NARS, este es el formato viaje, pero es que este tono, el Orgasm, es increíble. Es que tiene toques dorados y tal, no se te deja una mejilla preciosa. De colorete líquido no te lo pienses más, mi favorito es Rare Beauty, pero también tienes la otra alternativa, el de Giorgio Armani, pero este es un poquito más carito que este, así que este también te va a durarlo muchísimo si te quieres dar un caprichito o tal, los números nuevos de Giorgio Armani son una maravilla. El Beauty Like Bond de Charlotte Tilbury, si no te gusta en el formato esponjita te recomiendo los nuevos que han sacado de Giorgio, es que eso es una maravilla. Es que siento que es casi el mismo efecto, este potencia muchísimo más el color y este un poquito menos, pero ambos productos son una pasada. Solo que tener en cuenta que este se ensucia muchísimo, o sea muchísimo, y este de aquí es en formato corrector, controlas más cuánta cantidad de producto utilizas. Ahora que viene el veranito, el Benetim lo estoy utilizando muchísimo tanto para dar colorcito a los labios, y si no quieres llevar maquillaje y salir sin maquillaje, te echas un poquito esto de las mejillas y se ve un rojito muy natural, como que has tomado el sol y te has quemado ahí un poquillo. Máscara de pestañas, mi favorita es esta de Dior, es que te deja unos pestañones que flipa, yo creo que más de las que te deja la de Sky High de Maybelline, que está un súper viral. Y la Love the Leaf, la verdad que es que lo he amado y es que tenéis el formato pequeño y el formato grande por si queréis probarla. A mí me ha gustado muchísimo, tanto el cepillito es una maravilla y me dura todo el día. De esta también tenéis en formato waterproof. El gel fijador de cejas, amo el de Benefit, es una maravilla de mis primeros descubrimientos. También tenéis este de Anastasia de Erligir, ambos lo tenéis en mini talla por si queréis probarlo. Para rellenar las cejas me encanta muchísimo este rotulador de Benefit, siento que dibuja como pelo a pelo, es más natural, tienes en diferentes tonos, y este es el Brown Micro Filling Pen. Los labiales matte de Sephora duran una barbaridad. El rojo siento que es como un dupe del Defend the Beauty, este que deja aspecto aterciopelado. A mí me dura mucho, de hecho cuando estaba trabajando me suelen durar todo el día. Glosses que te hinchan los labios, tu face sin pensarlo. Y este de Dior, el Lip Maximizer, te deja unos labios súper bonitos, un color que siento que me dura muchísimo tiempo y es que obviamente el packaging me derrite. Deja el fijador, no lo pienses más, Charlotte Tilbury es la mejor opción. Y déjame saber si queréis que os diga más producto.</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>jirethmerchan</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>431800</v>
+      </c>
+      <c r="E200" t="n">
+        <v>7686</v>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuales fueron vuestras primeras compras? #parati #sephora #makeup #maquillaje </t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr"/>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>2024-06-03</t>
+        </is>
+      </c>
+      <c r="I200" t="n">
+        <v>92500</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@salmacadiz/video/7367379389044116768</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> soy la primera que para comprar algo siempre tiene que mirar recomendaciones en internet y sobre todo cuando estamos hablando de productos que precisamente no son muy baratos así que hoy vengo a daros mi opinión acerca de muchos virales de Sephora y bueno a contaros también un poquito de mi experiencia hoy se cumplen cuatro meses exactos de que me haya comprado todo esto que veis aquí si después de navidad cogí y me compré un montón de productos virales porque tenía muchas ganas de introducirlos en mi rutina de maquillaje a raíz de hacerme con muchos de ellos me he dado cuenta de que muchas cosas que comentan son ciertas pero muchas otras no lo son así que vamos con ello he decidido hacer grupos así que en este primer vídeo vamos a estar hablando de todos estos productos que veis aquí comenzamos con un esencial en mi rutina que es la bruma de sol de janeiro me encanta pero sí que es cierto que considero que los olores virales que son el 62 y el 59 son como muy típicos así que yo en el momento en el que olí la 71 me enamoré de hecho fue más perfecto porque dije la quiero aunque estamos hablando de un olor dulce no es un olor demasiado empalagoso es un olor que se nota la gente de mi alrededor siempre dice quién huele a galletas, quién huele a palomitas, quién huele a caramelo, quién huele también esos son los comentarios que recibo yo huele mucho, huele muy bien pero no es demasiado pesado ya os digo que yo la llevo y por ejemplo a mí no me levanta dolor de cabeza llevarla si vuestra pregunta es si dura, sí, este olor permanece en el tiempo yo me la suelo poner por la mañana al ducharme y a las 4 dentro de clase y a las 4 de la tarde la gente me dice que bien huele así que huele bien y dura tenéis diferentes tamaños este es el pequeño y como podéis ver os digo creo que son unos 90 mililitros de capacidad tengo que decir que dura muchísimo llevo más o menos unos 3 meses y medio probándola y bueno incluyéndola en mi rutina diariamente varias veces al día incluso y a mí me encanta pero cuesta unos 24 euros así que si os apetece cogeros el formato pequeñito para empezar yo os recomiendo esta opción porque es muy buena en cuanto a packaging perfecto el tapón es grande por lo que no se pierde y no permite fugas a la vez de que el flip-flip de toda la vida es la mejor opción a mí me encanta seguimos con Laneige este pack de 4 productos de la marca me costó un total de 25 euros tengo que decir que obviamente son mini tallas pero aparte de que son súper útiles para viajar ya sabéis que a mí me encantan son una forma muy muy guay de probar un producto sin necesidad de gastarte el dineral que puede llegar a costarte un tamaño original del mismo así que yo siempre os recomiendo que si estáis dudando entre compraros algo o no primero miréis a ver si hay mini tallas el tónico la verdad que no lo he probado porque yo no cambio el mío por nada y sí que es cierto que aunque me gusta ir introduciendo productos nuevos en mi rutina no he tenido la oportunidad de que me surja ningún viaje a raíz de ese momento así que este todavía no lo he probado vamos con otros tres productos la marca yo creo que se ha hecho muy viral sobre todo por esta mascarilla de labio que es una mascarilla hidratante para la noche obviamente se ponen los labios y yo creo que está sobrevalorada o sea es muy buen producto si me lo volvería a comprar si me encanta como sabe el olor la textura el efecto que deja si pero la gente lo pinta como si fuese algo único y realmente yo ya he tenido unos efectos muy muy parecidos con otro tipo de productos de otras marcas que no lo estoy discriminando pero sí que estoy diciendo que oye tanto hype pues yo creo que no merece otra cosa mala que tengo que decir de los aplicadores de la neige a pesar de que a mí el packaging me encanta porque son súper monos he de decir que a la hora de coger producto es muy difícil porque aunque sea la mini talla creo que debería de venir todo tipo de producto de la marca con el mismo formato acompañado de una espátula o algo para aplicarlo porque meter el dedo es poco higiénico que si siguiendo con la mascarilla de noche pienso un poco lo mismo es muy buena así que es cierto que me gusta muchísimo más que otras mascarillas hidratantes que hay para por la noche así que yo creo que tendré que seguir probándola porque está le he probado momentos más puntuales pero mi gran sorpresa con la marca ha sido la crema hidratante se llama water bank y os aseguro que hidrata mogollón sin necesidad de ser ni grasa ni untuosa ni pesada sientes la piel hidratada pero también con firmeza y elasticidad es como el equilibrio perfecto a mí me encanta llevo utilizándola un montón de meses y no me ha sacado granos de momento damos paso a otro viral el tónico de sandía de glow recipe y tengo que deciros que me encanta o sea es el tónico del que antes os he hablado no me despego de él porque realmente yo nunca usaba tónicos pero este me deja un aspecto de piel jugosa de piel sana de piel fresca una sensación de piel también suave me flipa sí que es cierto que bueno estéticamente es precioso yo no soy muy fanática del rosa pero es precioso es bote de cristal son 150 mililitros que llevo utilizando cuatro meses da para mucho pero bueno te viene con un seguro una especie como de pequeño taponcito para evitar que haya fugas del producto porque si no sí que se sale y bueno mientras lo tengas bien asegurado y no tires la tapita de arriba este producto no te tiene por qué dar ningún problema ahora bien hablemos del olor a mí me gusta el olor fresco esto huele a sandía pero para mí personalmente no me huele a la fruta me huele a la planta más que a la fruta sí huele bien pero es un olor muy muy potente es algo muy característico de la marca entonces si sois personas un poco aprensivas con olores yo recomiendo que antes de comprarlo porque vale 40 euros paséis por caja y os dejen no sé una muestra probar un tester cualquier cosa porque esto de verdad que huele muy fuerte y por último las famosísimas gotas iluminadoras de trunk elefante que tengo que decir que de las tres de las rosas las bronceadoras que son las marrones y de estas son mis favoritas sin lugar a duda esto se lo recomendaría hasta mi peor enemigo o sea de verdad son una pasada no me extraña el hype empiezo diciendo porque me gustan me gustan por el packaging porque son muy buenas y ya sabéis que yo soy como una ahorraca todo lo dorado me flipa luego sí que es cierto que pensaba que por el tamaño que tenían no iban a cundir porque cuestan 40 euros pero realmente cunden una barbaridad llevo usando las cuatro meses todos los días me maquillo no me maquille y es que queda un montón pesa todavía el bote una barbaridad lo siguiente a comentar el efecto que prometen es de piel sana de piel radiante de piel brillante pero sin ser un acabado bombilla como digo yo esto lo consigues que quieres suavizar el brillo te aplicas polvos matificantes y listo que quieres dejar la piel glowy tal y como se lleva ahora esto es tu aliado perfecto para que parezca que tienes la piel más sana del mundo esto te aporta luminosidad y sobre todo vitalidad al rostro para mí es una auténtica pasada el efecto que consigue además de que no sólo la utilizo como pre base de maquillaje acompañado de otros productos sino que también muchas veces cuando no me quiero maquillar con el simple hecho de aplicarme unas gotitas ya te cambia la cara os la recomiendo 100% y aunque cuesten 40 euros y sea un bote chiquito yo personalmente pienso que merece la pena</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>salmacadiz</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>31000</v>
+      </c>
+      <c r="E201" t="n">
+        <v>86800</v>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estasson mis humildes opiniones con precios incluidos🩷🩷 Prontito la parte 2!!  #fyp #viral #sephora #makeup #sephorahaul #sephorarecommendation #recomendaciones #feedback #laneige #glowrecipe #drunkelephant #soldejaniero @SEPHORA España </t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr"/>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>2024-05-10</t>
+        </is>
+      </c>
+      <c r="I201" t="n">
+        <v>672500</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@alba.puertas/video/7442700801601998113</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ¿Tienes un novio y no sabes qué regalarla a tu chica? Ya te estás quedando en este vídeo Traigo mi opinión más sincera pero de corazón De los 10 productos de Sephora que me volvería a comprar 200.000 veces Vamos allá ¿Quieres tener la piel más sedosa que una sabanamos? El exfoliante de Rare Beauty Huele increíble Que la sensación al echártelo lo bonita que deja la piel, girl Para un pelo brillante, sedoso, maravilloso, mi dupla Si te haces mucho clean look, que yo sé que te cae el pelo Quieres que te crezca mucho más, mucho más denso Esta maravilla de aquí Si quieres ser un génesis de crastas, vale la pena Para tener el pelo más brillante que hayas visto en tu vida Esta aceita amor He probado ninguna aceita así en mi vida y nunca lo voy a cambiar Jamás, nunca te soltaré El desodorante de Sol de Janeiro Tiene muchísimo producto pero un montón No irrita nada la axila y huele increíble Me lo agradeceréis A los novios que me estáis viendo que tenéis que regalar algo a vuestras novia estas navidades No voy a decir nada, solo apreciar esto La paleta más bonita que he tenido jamás Tiene tonos fríos, tiene tonos cálidos Las sombras con gliter son espectaculares Con un poco que he cogido me ha dado para los dos ojos La paleta Icy Nude de Huda Beauty ¿Crees que tu maquillaje parezca un filtro? El primer Easy Blur de Huda Beauty Esto te borra hasta lo que no tienes O sea, los poros desaparecen Además, hace que el maquillaje se apriera mucho mejor a la piel Quiero cubrir bien la ojera pero no quiero que se me reseque No quiero que se me cuarte Este corrector de Fenty Beauty Hidrata muchísimo la ojera que yo la tengo súper reseca Deja un efecto precioso y de aquí no se me mueve Si eres chicas de la isla y queréis estar bronceadas todo el año Las gotas bronceadoras de Ulala de Benefit You know what I mean Es que encima brilla esto Y obviamente los hula pero en el tono caramel Es un tono más calido que los hula normal, eh Simplemente precioso Por aquí podéis ver cómo queda Terminamos por mis hijos la razón de mi existencia El mejor lip combo de la historia O sea, mirad estos labios Como lip liner el Pillow Talk de Charlotte Tilbury El gloss, el mejor gloss de todo Sephora Ninguno es que no se aprecia lo que brilla esto Es que es increíble Es que es increíble El tono si flirty de los Faux Feelers de Huda Beauty Por cierto, mandale este vídeo a esa persona Que crees que te regale algo de esto</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>alba.puertas</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>91000</v>
+      </c>
+      <c r="E202" t="n">
+        <v>11500</v>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>TOP 10 productos de Sephora ⭐️ #cr7 #messi #f1 || 🤳🏽 albaapuertas</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr"/>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>2024-11-29</t>
+        </is>
+      </c>
+      <c r="I202" t="n">
+        <v>150800</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@maxabrechtt/video/7196750838268775686</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Fui hacia afuera, me compré un montón de cosas, así que voy a hacer un unboxing en un cual no sé si me atrapo toda una parte pero... voy a intentar mostrar y explicar todo lo que me compré más que nada porque no me compré todo porque sí, como que averigué bastante, compare con otras marcas y nada, ya la conclusión de lo que me compré lo primero que me compré fue el... ¿cómo se llama? Flawless Filter de Charlotte Tilbury que es como una base... no es una base, supuestamente es una prebase que vos tipo... te la pones y no te cubre por completo pero... te deja como un terminado más glowy, que dicen que está muy bueno bueno, lo siguiente que me compré es el Kousas Concealer que es el corrector que usa Hailey, supuestamente averigué esta marca y está bastante buena porque es como mitad maquillaje, mitad skincare entonces es como... tiene cobertura media pero como que no te deja la piel como muy maquillada me compré 80 mil de estos sprays de Mario Adescu que los uso bastante y están muy buenos, son como... como para hidratar la piel yo me lo pongo tipo... antes de maquillarme o si no me maquillo no sé, como que después de la crema me lo pongo de Charlotte Tilbury también me compré el Airbrush Setting Spray que es para un fijador, te terminas maquillaje y te lo pones supuestamente te dura un montón el maquillaje así que lo voy a probar después me compré este Sun Glow Gel, se llama de Sey, es la marca son como unas gotitas, como glowy, que te pones antes de la base, antes de todo y son como tono bronceado, entonces es como un auto-broncente del momento o sea, te lo lavas después, proteja la piel como bronceada y glowy para hacer maquillaje dicen que está muy bueno y las de Drunk Elephant que están de moda pero comparé y estas son mejores después vi en un montón de lados... no me meten las uñas vi en un montón de lados Olaplex, que es una marca para el pelo yo tengo el pelo en la B y esto supuestamente es el número 3 es como un baño de crema o algo así, te pones una vez a la semana y dicen que es muy bueno estos creo que no me los compré desde fuera pero están en la bolsa me compré dos Lifter Gloss de Maybelline que estuvieron bastante en moda los probé, están buenos, tienen un olor como medio fuerte, como chocolate medio dulce así que si sos medio sensible a los olores no sé si son para vos bueno, no me entrato en una parte claramente, ha sido el 2 ah y lo que sí, si quieren saber el tono de lo que me compré o el número de lo que sea lo dejo por comentarios porque si no, postas no sean larguísimos</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>maxabrechtt</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>143900</v>
+      </c>
+      <c r="E203" t="n">
+        <v>45400</v>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#unboxing de Makeup🤍🖤                                     #haul #sephora </t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr"/>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>2023-02-05</t>
+        </is>
+      </c>
+      <c r="I203" t="n">
+        <v>478100</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@sisoymachis/video/7288820282360401194</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ¡Col de lo que compré en Sephora! Yo nunca había comprado nada en Sephora, como que sí había entrado, pero jamás había comprado nada. Y esta vez por fin puedo comprar algo en Sephora y estoy... primera vuelta. Después de esto, la verdad que en bancarrota solo puedo comer aire y agua el resto de mi vida porque... Tenemos el corrector más viral de Too Faced. Este me lo he recomendado un 100 veces y lo compré. Obviamente el highlight y el blusher Charlotte Tilbury. Ustedes ya saben cuál es, este es súper viral en TikTok. Vamos a probarlo, vamos a probarlo. No puede fallar mi lip oil Dior. Oigan, yo amaba este, yo me compré uno hace poquito. Lo amé y conseguí exactamente el mismo otra vez. Este gloves también de Fenty Beauty. Me pareció súper bonito cuando lo vi como en el tester. Lo compré. Esto es por los compactos de One Size. Esta marca es de un TikToker influencer súper viral acá en Estados Unidos. Yo lo amo y la verdad siempre que los usaré que la piel es súper chelita. Los compré también. Laramente me tuve que comprar el blush de Rare Beauty. Según todo el mundo, esto es lo mejor del mundo. Que no sé qué, qué sé más. No sé, no sé, seguí en el review, seguí en el review. También me compré este highlight en polvo. Oigan, solamente miren ese glow. Compré el highlight en crema. O como se dice, qué es esto, en líquido. De Rare Beauty. Yo lo vi en el probar y fui como... Guau, qué es eso. Creo que eso ya fue como todas las compras que hice, pero me dieron regalitos, así que les voy a mostrar. Me dio este que es el birthday kit. Y tal, como yo compré hace poquito, pero como... Te voy a dar un regalito. Me dieron este que es como un set de shampoos, cosas como para, saben, como travel size. Me lo dieron. Me dieron dos dry shampoos. Ese es cuando tengo como que los sucios y me lo quiero lavar. Uno aplica esto y salió para la calle. Un gloss transparente. Nunca se falta un gloss transparente. Esto que la verdad no sé, pero sí, esto que es como super viral, pero no sé qué es. Esta manilla de Rare Beauty que dice Unbrer, la verdad la amé. Esto que es como un mini blush de Rare Beauty. Y una mascara también de Rare Beauty. Y ya eso fue todo por mi haul de Sephora hoy. La verdad sí estoy en un baño grabando porque es como el único lugar que tengo privado. Estoy viendo muchos reviews de todos los books que compré porque esto me va a embacarrota. Esto me va a embacarrota. Por favor, denle like. Gracias. Chao.</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>sisoymachis</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>435600</v>
+      </c>
+      <c r="E204" t="n">
+        <v>27700</v>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cuáles son sus favs ????? han probado alguno ??? los leooooooo aaaaaaaa amo el maquillaje #makeup #haul #sephora </t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr"/>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>2023-10-11</t>
+        </is>
+      </c>
+      <c r="I204" t="n">
+        <v>194100</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@.kunno/video/7435095398135401784</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ¡JOL de mis compras que hice el día de hoy en Sephora! ¡Aww! Antes de todo hice una gran compra, así que me regalaron esta cosmetiquera divina, rosita, amo. Y esta tote bag, que me encantó porque tiene como estas florecitas pintadas a mano. ¡Cute! Nada que ver con Sephora, pero al ladito de Sephora, ahí en la plaza que fui, que se llama Punto Valle, aquí en Monterrey, había una tienda que se llama New Era, que venden así como un chorro de gorras y cosas así. Y esta me encantó porque es como de velvet negra. Y esta otra tiene como florecitas bordadas. Me encantó, aparte me combina con mi look de hoy. Demás. Lo primero es mi wrist tuck de mi K18. Esta mascarilla es una mascarilla que te dejas durante el día y te lo juro, si tú eres una persona que se colora el pelo como yo, esto te va a restaurar por completo tu cabellera. De hecho, una de estas es para mi mamá porque me la pidió, o sea es buenísima. Para viajes y para obviamente traer en la bolsa, con eso de que ya está próxima el invierno, yo tipo super me reseco el rostro, entonces mi Beauty Elixir de Kaudalie, ya saben que es lo máximo. Oh, es que esto de verdad es un must, un must. Mi wrist tuck de mis minis de Aveda. Esta mascarilla es buenísima, es una mascarilla intensamente restauradora de cabellos, de verdad es buenísima y me encanta que viene así en su mini porque ahorita se me aproximan varios viajes. Entonces quería llevar más sin mis shampoocitos. Esta también es buenísimo, la línea de Strengthing Shampoo Botanical Repair de Aveda. La verdad es que sí me ayuda mucho a restaurar y me encanta porque sí, o sea para viajes esto es súper práctico. Y está condicionado porque casi no uso, pero de repente cuando tengo como las puntas super secas, amo. Y es que fácilmente yo me podría quedar horas y horas y horas en la sección de minis ya cuando vas en el caminito hacia apagar la caja, o sea, ¡ay! ¡Qué barro! Absolute Repair Molecular de L'Oreal Paris, o sea este en específico que es la Living Mask, o sea una mascarilla que también te dejas durante el día, no saben lo que es, o sea, la amo. Lo amo, lo amo, lo amociones, lo amo, lo amo, lo amo, lo amo, lo amo, lo amo, lo amo, lo amo, lo amo. Lo amo. Mi corrector favorito que en realidad es este de Clinique en el tono Ivory, o sea se los juro que me encanta porque me super ilumina de hecho es el que traigo puesto y vean nada más lo bonito que se ve y me encanta porque trae aquí como su esponjita, o sea también re-stuck. Estos parchesitos para ojo de Peter Thomas Rod, a mí me gustan mucho, por ejemplo cuando voy en el avión me los pongo o de repente en la noche que me toca como editar videos y me voy a quedar un rato en celular, me los aplico y se secan y aparte sí, o sea... ¿Calidad? ¿Calidad? Porque el precio está elevado, pero la calidad también. De Anastasia Beverly Hills moría yo por un plumín que fuera del tono de mi ceja y este, o sea, está súper parecido como ahorita es que ya saben que yo me de coloro, entonces me fascinó porque es como un lapicito que pinta así como rubio. Pues ni tan rubio, amiga, me habré equivocado. Ay, no me equivoqué. Creo que voy a quejarme con Sephora. O sea, ¿ustedes creen que este tono que viene aquí es este de mi ceja café? No. No. O sea, no es este tono. Aquí dice que es este tono y ¿por qué esto pinto a café? Bueno, lo que sí es que el gel para cejas también me dijeron que era buenísimo. Exactamente este brillosito que dice que es el Gel As Orseals Inco... O sea, que no tiene color, pero se supone que te deja así laminado, laminado, laminado, laminadísimo. O sea, laminadisísimo. Y sí, vean, bello. Vi que Elf acaba de sacar su colaboración con los vasos grandotes de Stan Lee y que de hecho hubo una polémica muy grande porque la gente compró como el puro agarrador de lip gloss y no de que el vaso completo. Pero pues dije, si sacaron esa colaboración por los glosses, supongo que va a ser muy bueno, ¿no? Vamos a ver. Sí, me fascinó. Este blush de Noot Stick en definitiva fue una recomendación de una amiga personal y me encantó. Este es el tono Hot Fire, pero vean, de un lado trae el ruborcito lindo, lindo. Yo lo agarré en este tono rojo porque vi que una persona que maquillaba a las ángeles de Victoria's Secret, a los ángeles de Victoria's Secret, decía que el rubor natural era el rojo porque nuestra sangre es roja, entonces si quieres un rubor natural, tienes que usar rubor rojo. Y sí, la verdad es que sí se ve súper lindo. Vean nada más, amo que trae su brochita aquí atrás. Esto es súper cool porque así no tienes que usar los dedos. Digo que a mí también me encanta usar los dedos, pero pues está bien. Y ya por último, pero no menos importante, amo, amo, amo, porque uno de mis polvos favoritos de la vida son los de Laura Mercier, pero hagan de cuenta que sacaron unos polvos que no traían como su bolita. Y ahorita en Sephora puedes encontrar como el kit de Navidad que sí trae como la bolita de regalo, o sea, viene así. Dejenme lo abro. Vean qué cool, trae su bolita y aquí está mi polvito. Yo este lo compré en el tono translucent. Es que no saben lo que es, o sea, de verdad, el efecto filtro. Me encanta que esté grandote. Nos vamos a poner un poquito porque si me siento brillosito, sobre todo aquí en esta zona, pero vean nada más. Dios, vital como filtro. No hay filtro alguno. Amo.</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>.kunno</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>32700000</v>
+      </c>
+      <c r="E205" t="n">
+        <v>39600</v>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">😍 Mi terapia: </t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr"/>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>2024-11-09</t>
+        </is>
+      </c>
+      <c r="I205" t="n">
+        <v>538200</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>